<commit_message>
Deploy 9e88182: import brings product pictures and warranty terms
</commit_message>
<xml_diff>
--- a/dist-admin/posfix-import-template.xlsx
+++ b/dist-admin/posfix-import-template.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Jobsheets" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Customers" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Products" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Warranty Terms" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -392,7 +393,7 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Current point balance. Whole number.</t>
+        <t>Optional. Current point balance, e.g. 12 or 1.75.</t>
       </text>
     </comment>
   </commentList>
@@ -453,6 +454,31 @@
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Yes = stock goes down on each sale.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Optional. A picture as data:image/... (what an old POS export holds) or an https link.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>POSFIX</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>REQUIRED. The short name staff pick, e.g. Screen 3 Months.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>REQUIRED. The full terms printed on the customer's receipt.</t>
       </text>
     </comment>
   </commentList>
@@ -748,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -781,7 +807,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1. Each tab is one kind of record: Sales, Money Out, Jobsheets, Customers, Products.</t>
+          <t>1. Each tab is one kind of record: Sales, Money Out, Jobsheets, Customers, Products, Warranty Terms.</t>
         </is>
       </c>
     </row>
@@ -909,7 +935,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Shop details, logo, payment methods, warranty terms: set them in Settings.</t>
+          <t>Shop details, logo, payment methods: set them in Settings.</t>
         </is>
       </c>
     </row>
@@ -969,6 +995,13 @@
       <c r="A35" t="inlineStr">
         <is>
           <t>Products: One row per product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Warranty Terms: One row per warranty wording staff pick at checkout.</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1678,6 +1711,7 @@
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1731,6 +1765,11 @@
           <t>Stock Tracked</t>
         </is>
       </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
@@ -1775,6 +1814,7 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K2" s="8" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -1807,6 +1847,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="K3" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -1817,4 +1858,47 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Screen 3 Months</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>3 months against manufacturing defects. Excludes liquid and physical damage.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Deploy b84e585: import Suppliers tab
</commit_message>
<xml_diff>
--- a/dist-admin/posfix-import-template.xlsx
+++ b/dist-admin/posfix-import-template.xlsx
@@ -10,10 +10,11 @@
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sales" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Money Out" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Jobsheets" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Customers" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Products" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Warranty Terms" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Suppliers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Jobsheets" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Customers" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Products" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Warranty Terms" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -303,67 +304,22 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>REQUIRED. Your old case / job number.</t>
+        <t>REQUIRED. As written in Money Out's Category / Supplier.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>REQUIRED. YYYY-MM-DD the device came in.</t>
+        <t>REQUIRED. purchase = a stock supplier. expense = everything else.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>REQUIRED.</t>
+        <t>Optional. cash or credit. Empty = cash.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>REQUIRED. Digits only.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. e.g. Phone, Laptop, Tablet.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>REQUIRED. What the customer reported.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>REQUIRED. new, progress, pendingPayment, complete or return.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Comma separated, e.g. Casing, Charger.</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. RM already paid. Numbers only.</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Staff name.</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Optional. YYYY-MM-DD HH:MM. Empty = the Date column.</t>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. YYYY-MM-DD HH:MM, for complete / return only.</t>
+        <t>Optional. Optional. A picture as data:image/... or an https link.</t>
       </text>
     </comment>
   </commentList>
@@ -378,22 +334,67 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>REQUIRED. Digits only. This is the customer's key.</t>
+        <t>REQUIRED. Your old case / job number.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
+        <t>REQUIRED. YYYY-MM-DD the device came in.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>REQUIRED.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>REQUIRED. Digits only.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. e.g. Phone, Laptop, Tablet.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>REQUIRED. What the customer reported.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
         <t>Optional.</t>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Ignored on upload: counted from Jobsheets. Kept so an Export file fits.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Current point balance, e.g. 12 or 1.75.</t>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>REQUIRED. new, progress, pendingPayment, complete or return.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Comma separated, e.g. Casing, Charger.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. RM already paid. Numbers only.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Staff name.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Optional. YYYY-MM-DD HH:MM. Empty = the Date column.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. YYYY-MM-DD HH:MM, for complete / return only.</t>
       </text>
     </comment>
   </commentList>
@@ -408,57 +409,22 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>REQUIRED.</t>
+        <t>REQUIRED. Digits only. This is the customer's key.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Type as text so leading zeros are kept.</t>
+        <t>Optional.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Optional.</t>
+        <t>Optional. Ignored on upload: counted from Jobsheets. Kept so an Export file fits.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Optional.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Should match a name in Money Out.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. RM you pay the supplier.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>REQUIRED. RM.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Quantity on hand.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Warn when stock falls to this.</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Yes = stock goes down on each sale.</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Optional. A picture as data:image/... (what an old POS export holds) or an https link.</t>
+        <t>Optional. Current point balance, e.g. 12 or 1.75.</t>
       </text>
     </comment>
   </commentList>
@@ -466,6 +432,71 @@
 </file>
 
 <file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>POSFIX</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>REQUIRED.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Type as text so leading zeros are kept.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Should match a name in Money Out.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. RM you pay the supplier.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>REQUIRED. RM.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Quantity on hand.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Warn when stock falls to this.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Yes = stock goes down on each sale.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Optional. A picture as data:image/... (what an old POS export holds) or an https link.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>POSFIX</author>
@@ -774,7 +805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -807,7 +838,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1. Each tab is one kind of record: Sales, Money Out, Jobsheets, Customers, Products, Warranty Terms.</t>
+          <t>1. Each tab is one kind of record: Sales, Money Out, Suppliers, Jobsheets, Customers, Products, Warranty Terms.</t>
         </is>
       </c>
     </row>
@@ -980,26 +1011,33 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jobsheets: One row per repair case.</t>
+          <t>Suppliers: Optional. One row per supplier or expense category, to give it a picture and cash/credit.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Customers: One row per customer. Points carry over their loyalty balance.</t>
+          <t>Jobsheets: One row per repair case.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Products: One row per product.</t>
+          <t>Customers: One row per customer. Points carry over their loyalty balance.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
+        <is>
+          <t>Products: One row per product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Warranty Terms: One row per warranty wording staff pick at checkout.</t>
         </is>
@@ -1407,6 +1445,75 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Parts Hub</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>purchase</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>credit</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Type" error="Pick one of: purchase, expense" type="list">
+      <formula1>"purchase,expense"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Payment" error="Pick one of: cash, credit" type="list">
+      <formula1>"cash,credit"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1617,7 +1724,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1692,7 +1799,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1860,7 +1967,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Deploy 911c703: import template Read Me
</commit_message>
<xml_diff>
--- a/dist-admin/posfix-import-template.xlsx
+++ b/dist-admin/posfix-import-template.xlsx
@@ -805,7 +805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -831,87 +831,83 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>HOW TO FILL IT</t>
+          <t>ONLY THIS FORMAT</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1. Each tab is one kind of record: Sales, Money Out, Suppliers, Jobsheets, Customers, Products, Warranty Terms.</t>
+          <t>POSFIX imports this template and nothing else. A file exported from another system will not upload as it is:</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2. Row 1 is the header. Do not rename, move or delete a header.</t>
+          <t>copy its columns into these tabs first, under these headers, in these formats.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>3. Red headers must be filled. Green headers may be left empty.</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>4. The grey rows under the header are EXAMPLES. Delete them before you upload.</t>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>THE SWITCH DAY</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5. Leave a tab empty (header only) if you have nothing for it.</t>
+          <t>1. Pick one day to move. Sell in the old system until the evening before, and in POSFIX from that morning.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>6. Hover or tap a header to read what goes in it.</t>
+          <t>2. Export from the old system at the end of its last day, so no sale is left behind.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>3. Never sell in both systems at once. A sale made in the old system after the export is not in POSFIX.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>FORMATS</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Dates: YYYY-MM-DD, e.g. 2026-01-31. Times: HH:MM, 24-hour, e.g. 14:30.</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>WHAT TO BRING</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Money: numbers only, e.g. 180 or 12.50. No 'RM', no commas.</t>
+          <t>Needed: Products (name, selling price, cost, stock), Customers and their points, Suppliers, open Jobsheets.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Phone: digits only, e.g. 0123456789. Spaces and dashes are removed on upload.</t>
+          <t>Optional: past Sales and Money Out, for your reports. Leave those tabs empty if you do not need them.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Yes / No and Type / Status columns: pick from the drop-down.</t>
+          <t>Not brought: old customer receipts and their links. Your customers open old receipts from the old system.</t>
         </is>
       </c>
     </row>
@@ -921,123 +917,275 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>SALES</t>
+          <t>STOCK</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>One row per item. A receipt with three items is three rows with the same Receipt No.</t>
+          <t>Count the stock on the shelf on the switch day and type that number in Products &gt; Stock.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Total is the row's amount (qty x unit price), not the whole receipt.</t>
+          <t>A number copied from the old system is often wrong, and POSFIX starts from whatever you type.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Old receipt numbers are kept for reference. New sales in POSFIX get POSFIX numbers.</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr"/>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>PICTURES</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>NOT IN THIS FILE</t>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>The Image columns may stay empty. Take product pictures in POSFIX with the phone camera later,</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Staff: add them in Settings. Each needs a PIN and signs in on their own phone.</t>
+          <t>fast sellers first. A product with no picture sells the same.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Shop details, logo, payment methods: set them in Settings.</t>
-        </is>
-      </c>
+      <c r="A25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>HOW TO FILL IT</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>TIP</t>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>1. Each tab is one kind of record: Sales, Money Out, Suppliers, Jobsheets, Customers, Products, Warranty Terms.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>A file from Settings &gt; Export Data uses the same headers, so its columns can be pasted straight in.</t>
+          <t>2. Row 1 is the header. Do not rename, move or delete a header.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>3. Red headers must be filled. Green headers may be left empty.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>4. The grey rows under the header are EXAMPLES. Delete them before you upload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>5. Leave a tab empty (header only) if you have nothing for it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>6. Hover or tap a header to read what goes in it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>FORMATS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Dates: YYYY-MM-DD, e.g. 2026-01-31. Times: HH:MM, 24-hour, e.g. 14:30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Money: numbers only, e.g. 180 or 12.50. No 'RM', no commas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Phone: digits only, e.g. 0123456789. Spaces and dashes are removed on upload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Yes / No and Type / Status columns: pick from the drop-down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>SALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>One row per item. A receipt with three items is three rows with the same Receipt No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Total is the row's amount (qty x unit price), not the whole receipt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Old receipt numbers are kept for reference. New sales in POSFIX get POSFIX numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>NOT IN THIS FILE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Staff: add them in Settings with the SAME names as in your old records, so their past sales stay theirs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Each needs a PIN and signs in on their own phone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Shop details, logo, payment methods: set them in Settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>UPLOADING AGAIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>A second upload replaces everything the last upload brought in, including any change made to it since.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Records keyed in at the counter are never touched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>WHAT EACH TAB HOLDS</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t>Sales: One row per ITEM sold. Several rows with the same Receipt No are one sale.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t>Money Out: One row per bill or purchase.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="57">
+      <c r="A57" t="inlineStr">
         <is>
           <t>Suppliers: Optional. One row per supplier or expense category, to give it a picture and cash/credit.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>Jobsheets: One row per repair case.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="59">
+      <c r="A59" t="inlineStr">
         <is>
           <t>Customers: One row per customer. Points carry over their loyalty balance.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="60">
+      <c r="A60" t="inlineStr">
         <is>
           <t>Products: One row per product.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>Warranty Terms: One row per warranty wording staff pick at checkout.</t>
         </is>

</xml_diff>